<commit_message>
Remove hard-coded API key and use environment variable
</commit_message>
<xml_diff>
--- a/syllabi_metadata.xlsx
+++ b/syllabi_metadata.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="60">
   <si>
     <t>Original name of syllabus PDF</t>
   </si>
@@ -70,68 +70,67 @@
     <t>Syllabus_topics_political_economy.pdf</t>
   </si>
   <si>
-    <t>Syllabus Fall 2025 Harvard Kennedy School of Government Harvard University</t>
-  </si>
-  <si>
-    <t>Econ 544: Political Economy and Institutions Professor Claudio Ferraz</t>
-  </si>
-  <si>
-    <t>The Logics of Violence: Rebels, Criminal Groups, and the State Fall 2025</t>
+    <t>Economic Development: Theory and Evidence</t>
+  </si>
+  <si>
+    <t>Political Economy and Institutions</t>
+  </si>
+  <si>
+    <t>The Logics of Violence: Rebels, Criminal Groups, and the State</t>
   </si>
   <si>
     <t>The Political Underpinnings of Prosperity and Poverty</t>
   </si>
   <si>
-    <t>2018 Political Economy of Development Political Science | Columbia University</t>
-  </si>
-  <si>
-    <t>Political Science 111 Principles of Political Science</t>
-  </si>
-  <si>
-    <t>Political Science 585 State Capacity</t>
-  </si>
-  <si>
-    <t>The Political Economy of Development PPHA41120/ECON35570/PLSC46600</t>
-  </si>
-  <si>
-    <t>ECONOM´ IA POL ´ ITICA</t>
-  </si>
-  <si>
-    <t>14.773: Political Economy of Institutions and Development</t>
-  </si>
-  <si>
-    <t>Topics in Political Economy Universitat de Barcelona</t>
-  </si>
-  <si>
-    <t>Eliana La Ferrara
-Office; La Ferrara</t>
-  </si>
-  <si>
-    <t>Claudio Ferraz
-Spring; Claudio Ferraz
-Office</t>
-  </si>
-  <si>
-    <t>Beatriz Magaloni e-mail</t>
-  </si>
-  <si>
-    <t>Leopoldo Fergusson Universidad de; Pablo Querub; James</t>
-  </si>
-  <si>
-    <t>Luis; My responsibility is to</t>
-  </si>
-  <si>
-    <t>Luis</t>
-  </si>
-  <si>
-    <t>the professors</t>
-  </si>
-  <si>
-    <t>esor</t>
-  </si>
-  <si>
-    <t>essors
-Daron Acemoglu</t>
+    <t>Political Economy of Development</t>
+  </si>
+  <si>
+    <t>Principles of Political Science</t>
+  </si>
+  <si>
+    <t>State Capacity</t>
+  </si>
+  <si>
+    <t>The Political Economy of Development</t>
+  </si>
+  <si>
+    <t>Economía Política</t>
+  </si>
+  <si>
+    <t>Political Economy of Institutions and Development</t>
+  </si>
+  <si>
+    <t>Topics in Political Economy</t>
+  </si>
+  <si>
+    <t>Eliana La Ferrara; Dani Rodrik</t>
+  </si>
+  <si>
+    <t>Claudio Ferraz</t>
+  </si>
+  <si>
+    <t>Beatriz Magaloni</t>
+  </si>
+  <si>
+    <t>Leopoldo Fergusson; Pablo Querubín; James A. Robinson</t>
+  </si>
+  <si>
+    <t>Macartan Humphreys</t>
+  </si>
+  <si>
+    <t>Luis R. Martinez</t>
+  </si>
+  <si>
+    <t>Chris Blattman; Eduardo Montero</t>
+  </si>
+  <si>
+    <t>Leopoldo Fergusson</t>
+  </si>
+  <si>
+    <t>Daron Acemoglu; Camilo Garcia-Jimeno</t>
+  </si>
+  <si>
+    <t>Leopoldo Fergusson; Dimitrios Xefteris</t>
   </si>
   <si>
     <t>2025</t>
@@ -155,39 +154,46 @@
     <t>2017</t>
   </si>
   <si>
-    <t>2008</t>
-  </si>
-  <si>
     <t>Fall</t>
   </si>
   <si>
     <t>Spring</t>
   </si>
   <si>
-    <t>Harvard Kennedy School of Government Harvard University</t>
-  </si>
-  <si>
-    <t>Cambridge University</t>
-  </si>
-  <si>
-    <t>University of Chicago jamesrobinson</t>
+    <t>Summer</t>
+  </si>
+  <si>
+    <t>Harvard University</t>
+  </si>
+  <si>
+    <t>University of British Columbia</t>
+  </si>
+  <si>
+    <t>Stanford University</t>
+  </si>
+  <si>
+    <t>Universidad de los Andes</t>
   </si>
   <si>
     <t>Columbia University</t>
   </si>
   <si>
-    <t>Principles of Political Science
-Emory University</t>
-  </si>
-  <si>
-    <t>State Capacity
-Emory University</t>
+    <t>Emory University</t>
+  </si>
+  <si>
+    <t>University of Chicago</t>
+  </si>
+  <si>
+    <t>Massachusetts Institute of Technology</t>
+  </si>
+  <si>
+    <t>Universitat de Barcelona</t>
+  </si>
+  <si>
+    <t>Lila</t>
   </si>
   <si>
     <t>Ricardy</t>
-  </si>
-  <si>
-    <t>Lila</t>
   </si>
 </sst>
 </file>
@@ -582,16 +588,16 @@
         <v>29</v>
       </c>
       <c r="D2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E2" t="s">
         <v>46</v>
       </c>
       <c r="F2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G2" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -605,16 +611,16 @@
         <v>30</v>
       </c>
       <c r="D3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E3" t="s">
         <v>47</v>
       </c>
       <c r="F3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="G3" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -628,13 +634,16 @@
         <v>31</v>
       </c>
       <c r="D4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E4" t="s">
         <v>46</v>
       </c>
+      <c r="F4" t="s">
+        <v>51</v>
+      </c>
       <c r="G4" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -648,13 +657,16 @@
         <v>32</v>
       </c>
       <c r="D5" t="s">
-        <v>40</v>
+        <v>41</v>
+      </c>
+      <c r="E5" t="s">
+        <v>48</v>
       </c>
       <c r="F5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G5" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -664,17 +676,20 @@
       <c r="B6" t="s">
         <v>22</v>
       </c>
+      <c r="C6" t="s">
+        <v>33</v>
+      </c>
       <c r="D6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G6" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -685,19 +700,19 @@
         <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E7" t="s">
         <v>47</v>
       </c>
       <c r="F7" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -711,16 +726,16 @@
         <v>34</v>
       </c>
       <c r="D8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E8" t="s">
         <v>47</v>
       </c>
       <c r="F8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G8" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -734,13 +749,16 @@
         <v>35</v>
       </c>
       <c r="D9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E9" t="s">
         <v>47</v>
       </c>
+      <c r="F9" t="s">
+        <v>55</v>
+      </c>
       <c r="G9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -754,13 +772,13 @@
         <v>36</v>
       </c>
       <c r="D10" t="s">
-        <v>43</v>
-      </c>
-      <c r="E10" t="s">
-        <v>46</v>
+        <v>44</v>
+      </c>
+      <c r="F10" t="s">
+        <v>52</v>
       </c>
       <c r="G10" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -774,13 +792,16 @@
         <v>37</v>
       </c>
       <c r="D11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E11" t="s">
         <v>47</v>
       </c>
+      <c r="F11" t="s">
+        <v>56</v>
+      </c>
       <c r="G11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -790,14 +811,17 @@
       <c r="B12" t="s">
         <v>28</v>
       </c>
-      <c r="D12" t="s">
-        <v>45</v>
+      <c r="C12" t="s">
+        <v>38</v>
       </c>
       <c r="E12" t="s">
-        <v>47</v>
+        <v>46</v>
+      </c>
+      <c r="F12" t="s">
+        <v>57</v>
       </c>
       <c r="G12" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Improved syllabus info extraction and added leaderboards for most cited and most recent syllabi across the set of analyzed syllabi
</commit_message>
<xml_diff>
--- a/syllabi_metadata.xlsx
+++ b/syllabi_metadata.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="69">
   <si>
     <t>Original name of syllabus PDF</t>
   </si>
@@ -34,126 +34,123 @@
     <t>University where this course was taught</t>
   </si>
   <si>
+    <t>New Syllabus Name</t>
+  </si>
+  <si>
     <t>Person in charge of digitizing this syllabus</t>
   </si>
   <si>
-    <t>DEV 101_ECON 2326_PED 101 - 2025 Fall (170665) (1).pdf</t>
-  </si>
-  <si>
-    <t>Econ 544 Syllabus 2021 Claudio Ferraz.pdf</t>
-  </si>
-  <si>
-    <t>Logics_Violence_Fall_2025_2-2.pdf</t>
-  </si>
-  <si>
-    <t>Los Andes 2020.pdf</t>
-  </si>
-  <si>
-    <t>PED_2018_syllabus.pdf</t>
-  </si>
-  <si>
-    <t>POLS 111 - Spring 2025 - Syllabus - v3.pdf</t>
-  </si>
-  <si>
-    <t>POLS 585 - State Capacity - Spring 2025 - Syllabus - v2.pdf</t>
-  </si>
-  <si>
-    <t>PPHA 41120_The Political Economy of Development_2024_Blattman Montero.pdf</t>
-  </si>
-  <si>
-    <t>Programa.pdf</t>
-  </si>
-  <si>
-    <t>Syllabus_6.pdf</t>
-  </si>
-  <si>
-    <t>Syllabus_topics_political_economy.pdf</t>
+    <t>Economic Development Theory and Evidence – Ferrara &amp; Rodrik – Fall 2025.pdf</t>
+  </si>
+  <si>
+    <t>Economía Política – Fergusson – Fall 2026.pdf</t>
+  </si>
+  <si>
+    <t>Political Economy and Institutions – Ferraz – Spring 2021.pdf</t>
+  </si>
+  <si>
+    <t>Political Economy of Development – Humphreys – Fall 2018.pdf</t>
+  </si>
+  <si>
+    <t>Political Economy of Institutions and Development – Acemoglu &amp; Garcia-Jimeno – Spring 2017.pdf</t>
+  </si>
+  <si>
+    <t>State Capacity – Martinez – Spring 2025.pdf</t>
+  </si>
+  <si>
+    <t>The Logics of Violence Rebels, Criminal Groups, and the State – Magaloni – Fall 2025.pdf</t>
+  </si>
+  <si>
+    <t>The Political Economy of Development – Blattman &amp; Montero – Spring 2023.pdf</t>
+  </si>
+  <si>
+    <t>The Political Underpinnings of Prosperity and Poverty – Fergusson &amp; Querubín &amp; Robinson – Summer 2020.pdf</t>
+  </si>
+  <si>
+    <t>Topics in Political Economy – Fergusson &amp; Xefteris – Fall.pdf</t>
   </si>
   <si>
     <t>Economic Development: Theory and Evidence</t>
   </si>
   <si>
+    <t>Economía Política</t>
+  </si>
+  <si>
     <t>Political Economy and Institutions</t>
   </si>
   <si>
+    <t>Political Economy of Development</t>
+  </si>
+  <si>
+    <t>Political Economy of Institutions and Development</t>
+  </si>
+  <si>
+    <t>State Capacity</t>
+  </si>
+  <si>
     <t>The Logics of Violence: Rebels, Criminal Groups, and the State</t>
   </si>
   <si>
+    <t>The Political Economy of Development</t>
+  </si>
+  <si>
     <t>The Political Underpinnings of Prosperity and Poverty</t>
   </si>
   <si>
-    <t>Political Economy of Development</t>
-  </si>
-  <si>
-    <t>Principles of Political Science</t>
-  </si>
-  <si>
-    <t>State Capacity</t>
-  </si>
-  <si>
-    <t>The Political Economy of Development</t>
-  </si>
-  <si>
-    <t>Economía Política</t>
-  </si>
-  <si>
-    <t>Political Economy of Institutions and Development</t>
-  </si>
-  <si>
     <t>Topics in Political Economy</t>
   </si>
   <si>
     <t>Eliana La Ferrara; Dani Rodrik</t>
   </si>
   <si>
+    <t>Leopoldo Fergusson</t>
+  </si>
+  <si>
     <t>Claudio Ferraz</t>
   </si>
   <si>
+    <t>Macartan Humphreys</t>
+  </si>
+  <si>
+    <t>Daron Acemoglu; Camilo Garcia-Jimeno</t>
+  </si>
+  <si>
+    <t>Luis R. Martinez</t>
+  </si>
+  <si>
     <t>Beatriz Magaloni</t>
   </si>
   <si>
+    <t>Chris Blattman; Eduardo Montero</t>
+  </si>
+  <si>
     <t>Leopoldo Fergusson; Pablo Querubín; James A. Robinson</t>
   </si>
   <si>
-    <t>Macartan Humphreys</t>
-  </si>
-  <si>
-    <t>Luis R. Martinez</t>
-  </si>
-  <si>
-    <t>Chris Blattman; Eduardo Montero</t>
-  </si>
-  <si>
-    <t>Leopoldo Fergusson</t>
-  </si>
-  <si>
-    <t>Daron Acemoglu; Camilo Garcia-Jimeno</t>
-  </si>
-  <si>
     <t>Leopoldo Fergusson; Dimitrios Xefteris</t>
   </si>
   <si>
     <t>2025</t>
   </si>
   <si>
+    <t>2026</t>
+  </si>
+  <si>
     <t>2021</t>
   </si>
   <si>
+    <t>2018</t>
+  </si>
+  <si>
+    <t>2017</t>
+  </si>
+  <si>
+    <t>2023</t>
+  </si>
+  <si>
     <t>2020</t>
   </si>
   <si>
-    <t>2018</t>
-  </si>
-  <si>
-    <t>2023</t>
-  </si>
-  <si>
-    <t>2026</t>
-  </si>
-  <si>
-    <t>2017</t>
-  </si>
-  <si>
     <t>Fall</t>
   </si>
   <si>
@@ -166,28 +163,58 @@
     <t>Harvard University</t>
   </si>
   <si>
+    <t>Universidad de los Andes</t>
+  </si>
+  <si>
     <t>University of British Columbia</t>
   </si>
   <si>
+    <t>Columbia University</t>
+  </si>
+  <si>
+    <t>Massachusetts Institute of Technology</t>
+  </si>
+  <si>
+    <t>Emory University</t>
+  </si>
+  <si>
     <t>Stanford University</t>
   </si>
   <si>
-    <t>Universidad de los Andes</t>
-  </si>
-  <si>
-    <t>Columbia University</t>
-  </si>
-  <si>
-    <t>Emory University</t>
-  </si>
-  <si>
     <t>University of Chicago</t>
   </si>
   <si>
-    <t>Massachusetts Institute of Technology</t>
-  </si>
-  <si>
     <t>Universitat de Barcelona</t>
+  </si>
+  <si>
+    <t>Economic Development: Theory and Evidence – Ferrara &amp; Rodrik – Fall 2025 – Harvard University</t>
+  </si>
+  <si>
+    <t>Economía Política – Fergusson – Fall 2026 – Universidad de los Andes</t>
+  </si>
+  <si>
+    <t>Political Economy and Institutions – Ferraz – Spring 2021 – University of British Columbia</t>
+  </si>
+  <si>
+    <t>Political Economy of Development – Humphreys – Fall 2018 – Columbia University</t>
+  </si>
+  <si>
+    <t>Political Economy of Institutions and Development – Acemoglu &amp; Garcia-Jimeno – Spring 2017 – Massachusetts Institute of Technology</t>
+  </si>
+  <si>
+    <t>State Capacity – Martinez – Spring 2025 – Emory University</t>
+  </si>
+  <si>
+    <t>The Logics of Violence: Rebels, Criminal Groups, and the State – Magaloni – Fall 2025 – Stanford University</t>
+  </si>
+  <si>
+    <t>The Political Economy of Development – Blattman &amp; Montero – Spring 2023 – University of Chicago</t>
+  </si>
+  <si>
+    <t>The Political Underpinnings of Prosperity and Poverty – Fergusson &amp; Querubín &amp; Robinson – Summer 2020 – Universidad de los Andes</t>
+  </si>
+  <si>
+    <t>Topics in Political Economy – Fergusson &amp; Xefteris – Fall – Universitat de Barcelona</t>
   </si>
   <si>
     <t>Lila</t>
@@ -551,10 +578,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -576,108 +603,123 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
         <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
+        <v>57</v>
+      </c>
+      <c r="H2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
         <v>19</v>
       </c>
       <c r="C3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G3" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="4" spans="1:7">
+      <c r="H3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
         <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E4" t="s">
         <v>46</v>
       </c>
       <c r="F4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
+        <v>59</v>
+      </c>
+      <c r="H4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5" t="s">
         <v>21</v>
       </c>
       <c r="C5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D5" t="s">
         <v>41</v>
       </c>
       <c r="E5" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G5" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
+        <v>60</v>
+      </c>
+      <c r="H5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
         <v>22</v>
       </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D6" t="s">
         <v>42</v>
@@ -686,38 +728,44 @@
         <v>46</v>
       </c>
       <c r="F6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G6" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
+        <v>61</v>
+      </c>
+      <c r="H6" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
         <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G7" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
+        <v>62</v>
+      </c>
+      <c r="H7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
         <v>24</v>
@@ -726,21 +774,24 @@
         <v>34</v>
       </c>
       <c r="D8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E8" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F8" t="s">
         <v>54</v>
       </c>
       <c r="G8" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
+        <v>63</v>
+      </c>
+      <c r="H8" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
       <c r="A9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B9" t="s">
         <v>25</v>
@@ -752,18 +803,21 @@
         <v>43</v>
       </c>
       <c r="E9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F9" t="s">
         <v>55</v>
       </c>
       <c r="G9" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
+        <v>64</v>
+      </c>
+      <c r="H9" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B10" t="s">
         <v>26</v>
@@ -774,16 +828,22 @@
       <c r="D10" t="s">
         <v>44</v>
       </c>
+      <c r="E10" t="s">
+        <v>47</v>
+      </c>
       <c r="F10" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="G10" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
+        <v>65</v>
+      </c>
+      <c r="H10" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B11" t="s">
         <v>27</v>
@@ -791,37 +851,17 @@
       <c r="C11" t="s">
         <v>37</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E11" t="s">
         <v>45</v>
-      </c>
-      <c r="E11" t="s">
-        <v>47</v>
       </c>
       <c r="F11" t="s">
         <v>56</v>
       </c>
       <c r="G11" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12" t="s">
-        <v>28</v>
-      </c>
-      <c r="C12" t="s">
-        <v>38</v>
-      </c>
-      <c r="E12" t="s">
-        <v>46</v>
-      </c>
-      <c r="F12" t="s">
-        <v>57</v>
-      </c>
-      <c r="G12" t="s">
-        <v>58</v>
+        <v>66</v>
+      </c>
+      <c r="H11" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>